<commit_message>
Crawlability audit: second verification round fixes
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/crawlability-amosziv-september-2026.xlsx
+++ b/public/crawlability-amosziv-september-2026.xlsx
@@ -501,7 +501,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>קישורים פנימיים לכתובות שמפנות (301/308): כתובת אחת (הבולטת: https://www.amosziv.co.il/טיפול-ביתי/, קישור נכנס אחד). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
+          <t>קישורים פנימיים ללא לוכסן סופי: 6 כתובות (הבולטת: https://www.amosziv.co.il/privacy-policy, 348 קישורים נכנסים). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>קישורים פנימיים ללא לוכסן סופי: 6 כתובות (הבולטת: https://www.amosziv.co.il/privacy-policy, 348 קישורים נכנסים). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
+          <t>קישורים פנימיים לכתובות שמפנות (301/308): כתובת אחת (הבולטת: https://www.amosziv.co.il/טיפול-ביתי/, קישור נכנס אחד). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>קישורי Cloudflare (ללא טיפול)</t>
+          <t>קישורים ללא צורך בטיפול (Cloudflare, הפניות לדומיין חיצוני)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">

</xml_diff>